<commit_message>
Add Test Data sheet to tcs.xlsx with the exact data used
One row per key used in Add to cart rows 41-42 and the Pre-Order Coverage
sheet: real value from the APP (or TO FILL), description, source and the
TC IDs that use it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YUiRueBr8ve5AHHG3UdcTU
</commit_message>
<xml_diff>
--- a/test-cases/tcs.xlsx
+++ b/test-cases/tcs.xlsx
@@ -9,6 +9,7 @@
     <sheet name="mystc5 OnePool Automation Cover" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="mystc5 Add to cart Automation" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Pre-Order Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Test Data" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -71,7 +72,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +89,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -159,6 +165,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8759,4 +8768,826 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Real value in APP</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Description / required state</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Used in TC IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>PUBLIC_USER</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Public user (not logged in)</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Continue as public user; no login</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>OP4</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-001, COMINGSOON-UI-005, COMINGSOON-UI-006, COMINGSOON-UI-007, COMINGSOON-UI-008, COMINGSOON-UI-009, COMINGSOON-UI-010, COMINGSOON-UI-011, COMINGSOON-UI-012, COMINGSOON-UI-014, COMINGSOON-UI-018, COMINGSOON-UI-022, COMINGSOON-UI-023, COMINGSOON-UI-029, COMINGSOON-UI-031, PREORDER-UI-001, PREORDER-UI-007, PREORDER-UI-010</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>LOGIN_USER_PRIMARY</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>504563459</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Full login (private user)</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>OP1</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>41, 42, COMINGSOON-UI-002, COMINGSOON-UI-005, COMINGSOON-UI-007, COMINGSOON-UI-009, COMINGSOON-UI-010, COMINGSOON-UI-012, COMINGSOON-UI-013, COMINGSOON-UI-014, COMINGSOON-UI-015, COMINGSOON-UI-016, COMINGSOON-UI-017, COMINGSOON-UI-018, COMINGSOON-UI-019, COMINGSOON-UI-023, COMINGSOON-UI-024, COMINGSOON-UI-026, COMINGSOON-UI-027, COMINGSOON-UI-028, COMINGSOON-UI-030, COMINGSOON-UI-031, COMINGSOON-UI-032, COMINGSOON-UI-033, PREORDER-UI-001, PREORDER-UI-002, PREORDER-UI-003, PREORDER-UI-004, PREORDER-UI-008, PREORDER-UI-012, PREORDER-UI-013, PREORDER-UI-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>OTP_USER_PRIMARY</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>504563459</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>OTP login with primary number</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>OP7</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-003, COMINGSOON-UI-020, COMINGSOON-UI-025, PREORDER-UI-005, PREORDER-UI-009</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>OTP_USER_SECONDARY</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>0507127863</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>OTP login with secondary number - limited access</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>OP8 / OP13</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-004, COMINGSOON-UI-006, COMINGSOON-UI-009, COMINGSOON-UI-010, COMINGSOON-UI-011, COMINGSOON-UI-021, COMINGSOON-UI-030, PREORDER-UI-001, PREORDER-UI-006, PREORDER-UI-011</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>DEV_NORMAL_INSTOCK</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>WHOOP PEAK BAND 5.0</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Normal in-stock device, Wearables category</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>User (Add to cart #36)</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-005, PREORDER-UI-012, PREORDER-UI-013</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>DEV_PARTIAL_OOS</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>PLUS 6TH</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Smart phones; Variation A out of stock, Variation B in stock</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>DEV_FREE_DEVICE</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>PLUS 6TH</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Smart phones; supports Free Device option</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>ELIGIBLE_VOICE_POSTPAID</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>504563459</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Line with active offer, used for Free Device</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_TIMER</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon = Y, releaseDate = now + 2d 03h 00m, price set</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>MS-2314 / MS-4095</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-010, COMINGSOON-UI-011, COMINGSOON-UI-015, COMINGSOON-UI-017, COMINGSOON-UI-018, COMINGSOON-UI-019, COMINGSOON-UI-020, COMINGSOON-UI-021, COMINGSOON-UI-022, COMINGSOON-UI-024, COMINGSOON-UI-025, COMINGSOON-UI-026, COMINGSOON-UI-027, COMINGSOON-UI-028, COMINGSOON-UI-032</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_NODATE</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon = Y, releaseDate empty/null, price set</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>MS-2314 P4</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-009, COMINGSOON-UI-018, COMINGSOON-UI-019, COMINGSOON-UI-020, COMINGSOON-UI-022</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_LT1DAY</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon = Y; releaseDate = now + 5h / + 120d / + 2 min (DEV_CS_SHORT purchasable after release)</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>MS-4095</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-012</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_FAR</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon = Y; releaseDate = now + 5h / + 120d / + 2 min (DEV_CS_SHORT purchasable after release)</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>MS-4095</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-013</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_SHORT</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon = Y; releaseDate = now + 5h / + 120d / + 2 min (DEV_CS_SHORT purchasable after release)</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>MS-4095</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-014, COMINGSOON-UI-016</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_NOPRICE</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon = Y, price null AND cashPrice null</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>MS-2314 P8</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-029, COMINGSOON-UI-030, COMINGSOON-UI-031</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_CASHONLY</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon = Y, price null, cashPrice set</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>MS-2314 P8</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-033</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_SOON_TAG_PRICE</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Store tag = soon with price set / price null</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>MS-2314 P2</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-001, COMINGSOON-UI-002, COMINGSOON-UI-003, COMINGSOON-UI-004, COMINGSOON-UI-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_SOON_TAG_NOPRICE</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Store tag = soon with price set / price null</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>MS-2314 P2</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_FLAG_NULL</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon empty/null, in stock</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>MS-2314 P3</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-023</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>DEV_PREORDER</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Pre-order device; NOSTOCK = stock 0 and pre-order enabled</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>OP24</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>PREORDER-UI-001, PREORDER-UI-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>DEV_PREORDER_NOSTOCK</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Pre-order device; NOSTOCK = stock 0 and pre-order enabled</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>OP24</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>PREORDER-UI-004, PREORDER-UI-005, PREORDER-UI-006, PREORDER-UI-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>DEV_PREORDER_SHORT</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>isPreOrder = Y; releaseDate now + 10d / now + 2 min / quantity &gt; 0</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>MS-4095 P5, Add to cart #34</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>PREORDER-UI-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>DEV_PREORDER_INSTOCK</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>isPreOrder = Y; releaseDate now + 10d / now + 2 min / quantity &gt; 0</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>MS-4095 P5, Add to cart #34</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>PREORDER-UI-008, PREORDER-UI-009, PREORDER-UI-010, PREORDER-UI-011, PREORDER-UI-012, PREORDER-UI-013</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>DEV_CS_AND_PREORDER</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>TO FILL</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>comingSoon = Y and isPreOrder = Y</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>PREORDER-UI-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Timer setup note</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Env</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>releaseDate values are relative to test start: set them in the test environment right before the run so timer assertions stay deterministic</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>MS-4095</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>COMINGSOON-UI-010, COMINGSOON-UI-011, COMINGSOON-UI-012, COMINGSOON-UI-013, COMINGSOON-UI-014, COMINGSOON-UI-015, COMINGSOON-UI-016, COMINGSOON-UI-017, COMINGSOON-UI-018, COMINGSOON-UI-019, COMINGSOON-UI-020, COMINGSOON-UI-021, COMINGSOON-UI-022, COMINGSOON-UI-024, COMINGSOON-UI-025, COMINGSOON-UI-026, COMINGSOON-UI-027, COMINGSOON-UI-028, COMINGSOON-UI-032</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rewrite template Test Data column in short User/Category/Device format
OnePool OP1-OP28 and Add to cart 1-42 now list only the data needed to run
each case, using real APP values (504563459, 0507127863, WHOOP PEAK BAND
5.0, PLUS 6TH, iPhone 17 Pro Max, IP16PRO and AWS10 MMax 24M,
test@stc.com.sa). Unknown products are marked TO FILL.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YUiRueBr8ve5AHHG3UdcTU
</commit_message>
<xml_diff>
--- a/test-cases/tcs.xlsx
+++ b/test-cases/tcs.xlsx
@@ -562,9 +562,11 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cash
+DPP: Not selected</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -637,9 +639,11 @@
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cash
+DPP: Selected</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
@@ -714,11 +718,11 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User
--with Get onepool Availability For A User, 
-quantity:0</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock 0)
+Purchase option: Cash
+DPP: Selected</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
@@ -782,8 +786,10 @@
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability
--Get onePool Device Availability (Public) --&gt; quantity&gt;0</t>
+          <t>User: Public user
+Category: Wearables
+Device: 6th device in Wearables (OnePool device: local stock 0) - public OnePool stock &gt; 0
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
@@ -848,8 +854,10 @@
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability
--Get onePool Device Availability (Public) --&gt; quantity:0</t>
+          <t>User: Public user
+Category: Wearables
+Device: 6th device in Wearables (OnePool device: local stock 0) - public OnePool stock 0
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
@@ -910,8 +918,10 @@
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">-"quantity": "1", "isOnePool": "N", in Get Device Availability
-</t>
+          <t>User: Public user
+Category: Wearables
+Device: 6th device in Wearables (fake OnePool: local stock 1, not OnePool)
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I7" s="1" t="inlineStr">
@@ -972,7 +982,10 @@
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: 504563459 (OTP login primary)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I8" s="1" t="inlineStr">
@@ -1050,7 +1063,10 @@
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: 0507127863 (OTP login secondary)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I9" s="1" t="inlineStr">
@@ -1129,9 +1145,12 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Installment
+Line: voice postpaid number (TO FILL)
+DPP: Not selected</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1220,9 +1239,12 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Installment
+Line: landline postpaid number (TO FILL)
+DPP: Selected</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -1310,7 +1332,10 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: Public user
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Installment</t>
         </is>
       </c>
       <c r="I12" s="1" t="inlineStr">
@@ -1384,7 +1409,11 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: 504563459 (OTP login primary)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Installment
+Line: voice postpaid number (TO FILL)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1477,7 +1506,10 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: 0507127863 (OTP login secondary)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Installment</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -1559,9 +1591,12 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Free Device
+Line: 504563459 (voice postpaid, active offer)
+DPP: Not selected</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -1651,9 +1686,12 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Free Device
+Line: landline postpaid / FWA (TO FILL)
+DPP: Selected</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1743,7 +1781,10 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: Public user
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Free Device</t>
         </is>
       </c>
       <c r="I17" s="1" t="inlineStr">
@@ -1817,7 +1858,12 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: 504563459 (OTP login primary)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Free Device
+Line: landline postpaid (TO FILL)
+DPP: Selected</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1910,7 +1956,10 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: 0507127863 (OTP login secondary)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Free Device</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -1996,9 +2045,12 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cashback
+Line: cashback eligible number (TO FILL)
+DPP: Not selected</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -2083,9 +2135,12 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cashback
+Line: cashback eligible number (TO FILL)
+DPP: Selected</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -2170,9 +2225,10 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User</t>
+          <t>User: user with no cashback eligible number (TO FILL)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cashback</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -2243,7 +2299,12 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: 504563459 (OTP login primary)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cashback
+Line: cashback eligible number (TO FILL)
+DPP: Selected</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -2332,7 +2393,10 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>-"quantity": "0", "isOnePool": "Y", in Get Device Availability</t>
+          <t>User: 0507127863 (OTP login secondary)
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)
+Purchase option: Cashback</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2417,9 +2481,9 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-Select third device in smart phones, 504563459
--isPreOrder:Y, in get device rules on variations levels , quantity:0
-</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (pre-order variation: stock 0)</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2476,10 +2540,10 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-Select third device in smart phones, 504563459
--isOnePoolPlus:Y in get device rules
--"quantity": &gt;"0", in Get Device Availability For A User
-</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (fake OnePool: local stock &gt; 0)
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I26" s="1" t="inlineStr">
@@ -2541,10 +2605,10 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-Select third device in smart phones, 504563459
--isOnePoolPlus:Y in get device rules
--"quantity": &gt;"0", in Get Device Availability For A User
-</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (fake OnePool: local stock &gt; 0)
+Purchase option: Installment</t>
         </is>
       </c>
       <c r="I27" s="1" t="inlineStr">
@@ -2607,10 +2671,10 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-Select third device in smart phones, 504563459
--isOnePoolPlus:Y in get device rules
--"quantity": &gt;"0", in Get Device Availability For A User
-</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (fake OnePool: local stock &gt; 0)
+Purchase option: Free Device</t>
         </is>
       </c>
       <c r="I28" s="1" t="inlineStr">
@@ -2673,11 +2737,10 @@
       </c>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>-Select third device in smart phones, 504563459
--isOnePoolPlus:Y, in get device rules on variations levels
--"quantity": "0", "isOnePool": "Y", in Get Device Availability For A User
--with Get onepool Availability For A User,  quantity:2
--device have partnership email</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: iPhone 16 Plus (OnePool device, OnePool stock 2, partnership device)
+Partnership email: test@stc.com.sa</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
@@ -2845,11 +2908,10 @@
       </c>
       <c r="H2" s="14" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Normal smartphone eligible for Add to Cart
-Get Device Availability For A User: quantity &gt; 0, isOnePool = N
-Purchase option: Cash
-Variation: Available color/storage</t>
+          <t>User: 504563459
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
@@ -2912,11 +2974,9 @@
       </c>
       <c r="H3" s="14" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Normal Add-to-Cart eligible smartphone supporting installment option
-Get Device Availability For A User: quantity &gt; 0, isOnePool = N
-DPP: Available
-Variation: Available</t>
+          <t>User: 504563459
+Device: TO FILL (supports Installment and DPP, in stock)
+DPP: Selected</t>
         </is>
       </c>
       <c r="I3" s="11" t="inlineStr">
@@ -2978,11 +3038,10 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Normal smartphone supporting installment
-Get Device Availability For A User: quantity &gt; 0, isOnePool = N
-Eligible postpaid line
-Installment plan available</t>
+          <t>User: 504563459
+Device: TO FILL (supports Installment, in stock)
+Purchase option: Installment
+Line: voice postpaid number (TO FILL)</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
@@ -3045,10 +3104,11 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Normal device supporting Free Device option
-Get Device Availability For A User: quantity &gt; 0, isOnePool = N
-Eligible postpaid/landline/FWA line with active offer</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: PLUS 6TH
+Purchase option: Free Device
+Line: 504563459</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
@@ -3109,10 +3169,10 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Normal device supporting Cashback
-Get Device Availability For A User: quantity &gt; 0, isOnePool = N
-Cashback eligible number available</t>
+          <t>User: 504563459
+Device: TO FILL (supports Cashback, in stock)
+Purchase option: Cashback
+Line: cashback eligible number (TO FILL)</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -3171,10 +3231,8 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Device supporting Cashback
-No cashback eligible numbers
-Get Device Availability For A User: quantity &gt; 0, isOnePool = N</t>
+          <t>User: user with no cashback eligible number (TO FILL)
+Device: TO FILL (supports Cashback)</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
@@ -3229,10 +3287,9 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>User: Not logged in
-Device: Normal available device
-Public device availability: quantity &gt; 0
-isOnePool = N</t>
+          <t>User: Public user
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -3292,10 +3349,9 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Primary MSISDN: 504563459
-Device: Normal Add-to-Cart eligible device
-quantity &gt; 0
-isOnePool = N</t>
+          <t>User: 504563459 (OTP login primary)
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
@@ -3353,11 +3409,9 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Secondary MSISDN: 0507127863
-Device: Normal device
-quantity &gt; 0
-isOnePool = N
-Secondary line eligibility must be checked</t>
+          <t>User: 0507127863 (OTP login secondary)
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
@@ -3416,10 +3470,9 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Normal non-OnePool device
-Get Device Availability For A User: quantity = 0, isOnePool = N
-isOnePoolPlus = N</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: IP16PRO and AWS10 MMax 24M (out of stock)</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
@@ -3476,10 +3529,10 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Normal non-OnePool device
-Get Device Availability For A User: quantity &gt; 0, isOnePool = N
-Available variation</t>
+          <t>User: 504563459
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -3537,11 +3590,9 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Third device in Smart Phones
-isOnePoolPlus = Y in Get Device Rules on variation level
-Get Device Availability For A User: quantity = 0, isOnePool = Y
-Get onePool Availability For A User: quantity &gt; 0</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
@@ -3598,10 +3649,9 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: OnePool device
-Get Device Availability For A User: quantity = 0, isOnePool = Y
-Get onePool Availability For A User: quantity = 0</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock 0)</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
@@ -3658,10 +3708,9 @@
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Device with isOnePoolPlus = Y in Get Device Rules
-Get Device Availability For A User: quantity &gt; 0
-Device should be processed as normal available inventory</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (fake OnePool: local stock &gt; 0)</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
@@ -3720,9 +3769,8 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device variation: quantity = 0
-Get Device Rules: isPreOrder = Y</t>
+          <t>User: 504563459
+Device: TO FILL (pre-order device: stock 0)</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
@@ -3779,11 +3827,9 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Add-to-Cart eligible device requiring partnership email
-quantity &gt; 0
-isOnePool = N
-Valid partnership email</t>
+          <t>User: 504563459
+Device: TO FILL (partnership device, in stock)
+Partnership email: test@stc.com.sa</t>
         </is>
       </c>
       <c r="I17" s="14" t="inlineStr">
@@ -3841,11 +3887,11 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Smartphone with at least 2 storage variations
-Storage A: quantity &gt; 0
-Storage B: quantity &gt; 0
-Purchase: Cash</t>
+          <t>User: 504563459
+Device: TO FILL (2 storages in stock)
+Storage A: TO FILL
+Storage B: TO FILL
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
@@ -3903,12 +3949,11 @@
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Smartphone with at least 2 colors
-Color A: quantity &gt; 0
-Color B: quantity &gt; 0
-Same storage
-Purchase: Cash</t>
+          <t>User: 504563459
+Device: TO FILL (2 colors in stock, same storage)
+Color A: TO FILL
+Color B: TO FILL
+Purchase option: Cash</t>
         </is>
       </c>
       <c r="I19" s="11" t="inlineStr">
@@ -3965,11 +4010,9 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Same device
-Variation A: quantity = 0
-Variation B: quantity &gt; 0
-isOnePool = N</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: PLUS 6TH (Variation A out of stock, Variation B in stock)</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
@@ -4027,10 +4070,10 @@
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Normal eligible device
-quantity &gt; 0
-Known color/storage/price</t>
+          <t>User: 504563459
+Cart: empty
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
@@ -4086,10 +4129,9 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device A: quantity &gt; 0, isOnePool = N
-Device B: quantity &gt; 0, isOnePool = N
-Both Add-to-Cart eligible</t>
+          <t>User: 504563459
+Device A: WHOOP PEAK BAND 5.0 (Wearables)
+Device B: iPhone 17 Pro Max (Smart phones)</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
@@ -4146,9 +4188,9 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Same normal device + same variation
-quantity sufficient for repeated action</t>
+          <t>User: 504563459
+Cart: 1 x WHOOP PEAK BAND 5.0
+Device: WHOOP PEAK BAND 5.0 (same variation)</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
@@ -4205,8 +4247,8 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-One or more normal devices already in Cart</t>
+          <t>User: 504563459
+Cart: WHOOP PEAK BAND 5.0, iPhone 17 Pro Max</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
@@ -4263,8 +4305,8 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Cart contains one or more Add-to-Cart eligible devices</t>
+          <t>User: 504563459
+Cart: WHOOP PEAK BAND 5.0, iPhone 17 Pro Max</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
@@ -4320,8 +4362,9 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Normal eligible device already added</t>
+          <t>User: 504563459
+Cart: 1 x WHOOP PEAK BAND 5.0
+Categories: Smart phones, Wearables</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
@@ -4376,10 +4419,10 @@
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Normal eligible device
-quantity &gt; 0
-Cash</t>
+          <t>User: 504563459
+Cart: empty
+Device: WHOOP PEAK BAND 5.0
+Taps: 5 within 1 second</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
@@ -4436,10 +4479,9 @@
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Normal eligible device
-Availability service: 500 or timeout
-Retry: success with quantity &gt; 0</t>
+          <t>User: 504563459
+Device: WHOOP PEAK BAND 5.0
+Network: OFF then ON</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
@@ -4500,10 +4542,8 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Normal eligible device
-Known product name/color/storage/price
-quantity &gt; 0</t>
+          <t>User: 504563459
+Cart: 1 x WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
@@ -4560,12 +4600,9 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Existing Cart item: Prepaid Order
-New Product: Any Add-to-Cart eligible product
-New Product quantity: &gt; 0
-isOnePool: N
-Purchase option: Cas</t>
+          <t>User: 504563459
+Cart: Prepaid order (TO FILL)
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
@@ -4629,11 +4666,9 @@
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Existing Cart Item: Normal Add-to-Cart eligible device
-Existing Device quantity: &gt; 0
-isOnePool: N
-New Item: Prepaid Order</t>
+          <t>User: 504563459
+Cart: 1 x WHOOP PEAK BAND 5.0
+New item: Prepaid order (TO FILL)</t>
         </is>
       </c>
       <c r="I31" s="11" t="inlineStr">
@@ -4698,12 +4733,9 @@
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Get User Cart Details: CART ITEM COUNT = X
-Existing Cart Items: X items
-New Product: Add-to-Cart eligible product
-New Product quantity: &gt; 0
-isOnePool: N</t>
+          <t>User: 504563459
+Cart: maximum allowed items (CART ITEM COUNT = X)
+Device: iPhone 17 Pro Max</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
@@ -4768,10 +4800,8 @@
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Product: Back Order device
-Device Rule API: RESERVABLE = "Y"
-Product Status: Back Order
+          <t>User: 504563459
+Device: TO FILL (back order, reservable)
 Action: Reserve Now</t>
         </is>
       </c>
@@ -4838,11 +4868,9 @@
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: OnePool eligible device
-Get Device Availability For A User: isOnePool = "Y"
-Local quantity: 0
-OnePool Availability: quantity &gt; 0</t>
+          <t>User: 504563459
+Category: Smart phones
+Device: 3rd device in Smart phones (OnePool device: local stock 0, OnePool stock &gt; 0)</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
@@ -4907,10 +4935,8 @@
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Pre Order eligible device
-Device Rule API: isPreOrder = "Y"
-Product Type: Pre Order</t>
+          <t>User: 504563459
+Device: TO FILL (pre-order device)</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
@@ -4974,12 +5000,10 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Existing Cart Item: Pre Order device
-Device Rule: isPreOrder = "Y"
-New Product: Normal available device
-New Device quantity: &gt; 0
-isOnePool: N</t>
+          <t>User: 504563459
+Cart: pre-order device (TO FILL)
+Category: Wearables
+Device: WHOOP PEAK BAND 5.0</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
@@ -5043,10 +5067,9 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Existing Cart Item: Normal device, quantity &gt; 0
-New Product: Pre Order device
-New Product Device Rule: isPreOrder = "Y"</t>
+          <t>User: 504563459
+Cart: 1 x WHOOP PEAK BAND 5.0
+Device: TO FILL (pre-order device)</t>
         </is>
       </c>
       <c r="I37" s="14" t="inlineStr">
@@ -5109,12 +5132,9 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Normal Add-to-Cart eligible device
-quantity: &gt; 0
-isOnePool: N
-STC Protect: Eligible/Available
-Selection: Add STC Protect</t>
+          <t>User: 504563459
+Device: TO FILL (STC Protect eligible, in stock)
+STC Protect: Selected</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
@@ -5179,12 +5199,9 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Same STC Protect eligible device
-quantity: &gt; 0
-isOnePool: N
-STC Protect: Available
-Selection: Continue without STC Protec</t>
+          <t>User: 504563459
+Device: TO FILL (STC Protect eligible, in stock)
+STC Protect: Not selected</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
@@ -5249,12 +5266,9 @@
       </c>
       <c r="H40" s="9" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Device: Add-to-Cart eligible Partnership device
-quantity: &gt; 0
-isOnePool: N
-Partnership: Enabled
-Email: Valid partnership email "test@stc.com.sa"</t>
+          <t>User: 504563459
+Device: TO FILL (partnership device, in stock)
+Partnership email: test@stc.com.sa</t>
         </is>
       </c>
       <c r="I40" s="9" t="inlineStr">
@@ -5318,10 +5332,8 @@
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>MSISDN: 504563459
-Product: Back Order device
-Device Rule API: RESERVABLE = "N"
-Product Status: Back Order</t>
+          <t>User: 504563459
+Device: TO FILL (back order, not reservable)</t>
         </is>
       </c>
       <c r="I41" s="9" t="inlineStr">
@@ -5386,6 +5398,7 @@
       <c r="H42" s="11" t="inlineStr">
         <is>
           <t>User: 504563459
+Category: Smart phones
 Device: PLUS 6TH (Variation A out of stock, Variation B in stock)</t>
         </is>
       </c>
@@ -5451,7 +5464,9 @@
       <c r="H43" s="11" t="inlineStr">
         <is>
           <t>User: 504563459
+Category: Smart phones
 Device: PLUS 6TH
+Purchase option: Free Device
 Line: 504563459</t>
         </is>
       </c>

</xml_diff>